<commit_message>
SqlType.xlsx: VECTOR 자료형 추가 (MySQL 9.0+, MariaDB 11.7+, PostgreSQL/pgvector, Oracle 23ai, SQL Server 2025)
</commit_message>
<xml_diff>
--- a/ermaster_plugin/src/main/resources/SqlType.xlsx
+++ b/ermaster_plugin/src/main/resources/SqlType.xlsx
@@ -75,7 +75,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +86,11 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00808080"/>
       </patternFill>
     </fill>
   </fills>
@@ -187,7 +192,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -252,6 +257,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -2568,7 +2574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ148"/>
+  <dimension ref="A1:CJ149"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="30.125" defaultRowHeight="14.25"/>
   <cols>
     <col width="36.625" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
@@ -26396,139 +26402,139 @@
       <c r="D136" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G136" t="inlineStr">
+      <c r="G136" s="0" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="R136" t="inlineStr">
+      <c r="R136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="S136" t="inlineStr">
+      <c r="S136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="T136" t="inlineStr">
+      <c r="T136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="U136" t="n">
-        <v>0</v>
-      </c>
-      <c r="V136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD136" t="inlineStr">
+      <c r="U136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AE136" t="inlineStr">
+      <c r="AE136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AF136" t="inlineStr">
+      <c r="AF136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AG136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ136" t="inlineStr">
+      <c r="AG136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AK136" t="inlineStr">
+      <c r="AK136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AL136" t="inlineStr">
+      <c r="AL136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AM136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP136" t="inlineStr">
+      <c r="AM136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AQ136" t="inlineStr">
+      <c r="AQ136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AR136" t="inlineStr">
+      <c r="AR136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AS136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW136" t="inlineStr">
+      <c r="AS136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW136" s="0" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="BB136" t="inlineStr">
+      <c r="BB136" s="0" t="inlineStr">
         <is>
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="BC136" t="inlineStr">
+      <c r="BC136" s="0" t="inlineStr">
         <is>
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="BH136" t="inlineStr">
+      <c r="BH136" s="0" t="inlineStr">
         <is>
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="BI136" t="inlineStr">
+      <c r="BI136" s="0" t="inlineStr">
         <is>
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="CF136" t="inlineStr">
+      <c r="CF136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="CG136" t="inlineStr">
+      <c r="CG136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="CH136" t="inlineStr">
+      <c r="CH136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="CI136" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ136" t="n">
+      <c r="CI136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ136" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -26547,68 +26553,68 @@
       <c r="D137" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G137" t="inlineStr">
+      <c r="G137" s="0" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="R137" t="inlineStr">
+      <c r="R137" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="S137" t="inlineStr">
+      <c r="S137" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AE137" t="inlineStr">
+      <c r="AE137" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AK137" t="inlineStr">
+      <c r="AK137" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AP137" t="inlineStr">
+      <c r="AP137" s="0" t="inlineStr">
         <is>
           <t>jsonb</t>
         </is>
       </c>
-      <c r="AQ137" t="inlineStr">
+      <c r="AQ137" s="0" t="inlineStr">
         <is>
           <t>jsonb</t>
         </is>
       </c>
-      <c r="AR137" t="inlineStr">
+      <c r="AR137" s="0" t="inlineStr">
         <is>
           <t>jsonb</t>
         </is>
       </c>
-      <c r="AS137" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT137" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW137" t="inlineStr">
+      <c r="AS137" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT137" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW137" s="0" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="BC137" t="inlineStr">
+      <c r="BC137" s="0" t="inlineStr">
         <is>
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="BI137" t="inlineStr">
+      <c r="BI137" s="0" t="inlineStr">
         <is>
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="CG137" t="inlineStr">
+      <c r="CG137" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
@@ -26793,7 +26799,7 @@
           <t>json</t>
         </is>
       </c>
-      <c r="AD139" t="inlineStr">
+      <c r="AD139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
@@ -26803,15 +26809,15 @@
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AF139" t="inlineStr">
+      <c r="AF139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AG139" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH139" t="n">
+      <c r="AG139" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH139" s="0" t="n">
         <v>0</v>
       </c>
       <c r="AK139" s="0" t="inlineStr">
@@ -26855,7 +26861,7 @@
           <t>nvarchar(max)</t>
         </is>
       </c>
-      <c r="CF139" t="inlineStr">
+      <c r="CF139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
@@ -26865,15 +26871,15 @@
           <t>multipoint</t>
         </is>
       </c>
-      <c r="CH139" t="inlineStr">
+      <c r="CH139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="CI139" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ139" t="n">
+      <c r="CI139" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ139" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -27155,46 +27161,46 @@
       <c r="AT143" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="BB143" t="inlineStr">
+      <c r="BB143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BC143" t="inlineStr">
+      <c r="BC143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BD143" t="inlineStr">
+      <c r="BD143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BE143" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF143" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH143" t="inlineStr">
+      <c r="BE143" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF143" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BI143" t="inlineStr">
+      <c r="BI143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BJ143" t="inlineStr">
+      <c r="BJ143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BK143" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL143" t="n">
+      <c r="BK143" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL143" s="0" t="n">
         <v>0</v>
       </c>
       <c r="CF143" s="0" t="inlineStr">
@@ -27373,7 +27379,7 @@
       <c r="BL145" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="CF145" t="inlineStr">
+      <c r="CF145" s="0" t="inlineStr">
         <is>
           <t>inet6</t>
         </is>
@@ -27383,15 +27389,15 @@
           <t>inet6</t>
         </is>
       </c>
-      <c r="CH145" t="inlineStr">
+      <c r="CH145" s="0" t="inlineStr">
         <is>
           <t>inet6</t>
         </is>
       </c>
-      <c r="CI145" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ145" t="n">
+      <c r="CI145" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ145" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -27411,25 +27417,25 @@
           <t>geometry</t>
         </is>
       </c>
-      <c r="AJ146" t="inlineStr">
+      <c r="AJ146" s="0" t="inlineStr">
         <is>
           <t>sdo_geometry</t>
         </is>
       </c>
-      <c r="AK146" t="inlineStr">
+      <c r="AK146" s="0" t="inlineStr">
         <is>
           <t>sdo_geometry</t>
         </is>
       </c>
-      <c r="AL146" t="inlineStr">
+      <c r="AL146" s="0" t="inlineStr">
         <is>
           <t>sdo_geometry</t>
         </is>
       </c>
-      <c r="AM146" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN146" t="n">
+      <c r="AM146" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN146" s="0" t="n">
         <v>0</v>
       </c>
       <c r="AP146" s="0" t="inlineStr">
@@ -27579,6 +27585,62 @@
       <c r="CG148" s="0" t="inlineStr">
         <is>
           <t>geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>java.lang.Object</t>
+        </is>
+      </c>
+      <c r="C149" t="b">
+        <v>1</v>
+      </c>
+      <c r="D149" t="b">
+        <v>0</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="K149" s="22" t="n"/>
+      <c r="Q149" s="22" t="n"/>
+      <c r="W149" s="22" t="n"/>
+      <c r="AD149" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AJ149" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AP149" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AU149" s="22" t="n"/>
+      <c r="BB149" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="BG149" s="22" t="n"/>
+      <c r="BM149" s="22" t="n"/>
+      <c r="BS149" s="22" t="n"/>
+      <c r="BY149" s="22" t="n"/>
+      <c r="CF149" t="inlineStr">
+        <is>
+          <t>vector</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix SqlType.xlsx: DBMS별 고유 자료형 Alias 및 Key 1:1 매핑 정비 (inet4/inet6/spatial/vector 충돌 해결)
</commit_message>
<xml_diff>
--- a/ermaster_plugin/src/main/resources/SqlType.xlsx
+++ b/ermaster_plugin/src/main/resources/SqlType.xlsx
@@ -2574,7 +2574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ149"/>
+  <dimension ref="A1:CJ147"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="30.125" defaultRowHeight="14.25"/>
   <cols>
     <col width="36.625" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
@@ -26398,145 +26398,92 @@
           <t>java.lang.String</t>
         </is>
       </c>
-      <c r="C136" s="9" t="n"/>
+      <c r="C136" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="D136" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="G136" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E136" s="22" t="n"/>
+      <c r="G136" s="0" t="n"/>
+      <c r="K136" s="22" t="n"/>
       <c r="R136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="S136" s="0" t="inlineStr">
+      <c r="S136" s="0" t="n"/>
+      <c r="T136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="T136" s="0" t="inlineStr">
+      <c r="U136" s="0" t="n"/>
+      <c r="V136" s="0" t="n"/>
+      <c r="W136" s="22" t="n"/>
+      <c r="AD136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="U136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="V136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD136" s="0" t="inlineStr">
+      <c r="AE136" s="0" t="n"/>
+      <c r="AF136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AE136" s="0" t="inlineStr">
+      <c r="AG136" s="0" t="n"/>
+      <c r="AH136" s="0" t="n"/>
+      <c r="AJ136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AF136" s="0" t="inlineStr">
+      <c r="AK136" s="0" t="n"/>
+      <c r="AL136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AG136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ136" s="0" t="inlineStr">
+      <c r="AM136" s="0" t="n"/>
+      <c r="AN136" s="0" t="n"/>
+      <c r="AP136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AK136" s="0" t="inlineStr">
+      <c r="AQ136" s="0" t="n"/>
+      <c r="AR136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AL136" s="0" t="inlineStr">
+      <c r="AS136" s="0" t="n"/>
+      <c r="AT136" s="0" t="n"/>
+      <c r="AU136" s="22" t="n"/>
+      <c r="AW136" s="0" t="n"/>
+      <c r="BA136" s="22" t="n"/>
+      <c r="BB136" s="0" t="n"/>
+      <c r="BC136" s="0" t="n"/>
+      <c r="BG136" s="22" t="n"/>
+      <c r="BH136" s="0" t="n"/>
+      <c r="BI136" s="0" t="n"/>
+      <c r="BM136" s="22" t="n"/>
+      <c r="BS136" s="22" t="n"/>
+      <c r="BY136" s="22" t="n"/>
+      <c r="CF136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AM136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP136" s="0" t="inlineStr">
+      <c r="CG136" s="0" t="n"/>
+      <c r="CH136" s="0" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="AQ136" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AR136" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AS136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW136" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="BB136" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BC136" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BH136" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BI136" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="CF136" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="CG136" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="CH136" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="CI136" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ136" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI136" s="0" t="n"/>
+      <c r="CJ136" s="0" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="9" t="inlineStr">
@@ -26549,76 +26496,47 @@
           <t>java.lang.String</t>
         </is>
       </c>
-      <c r="C137" s="9" t="n"/>
+      <c r="C137" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="D137" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="G137" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="R137" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="S137" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AE137" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AK137" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E137" s="22" t="n"/>
+      <c r="G137" s="0" t="n"/>
+      <c r="K137" s="22" t="n"/>
+      <c r="Q137" s="22" t="n"/>
+      <c r="R137" s="0" t="n"/>
+      <c r="S137" s="0" t="n"/>
+      <c r="W137" s="22" t="n"/>
+      <c r="AC137" s="22" t="n"/>
+      <c r="AE137" s="0" t="n"/>
+      <c r="AI137" s="22" t="n"/>
+      <c r="AK137" s="0" t="n"/>
       <c r="AP137" s="0" t="inlineStr">
         <is>
           <t>jsonb</t>
         </is>
       </c>
-      <c r="AQ137" s="0" t="inlineStr">
+      <c r="AQ137" s="0" t="n"/>
+      <c r="AR137" s="0" t="inlineStr">
         <is>
           <t>jsonb</t>
         </is>
       </c>
-      <c r="AR137" s="0" t="inlineStr">
-        <is>
-          <t>jsonb</t>
-        </is>
-      </c>
-      <c r="AS137" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT137" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW137" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="BC137" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BI137" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="CG137" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
+      <c r="AS137" s="0" t="n"/>
+      <c r="AT137" s="0" t="n"/>
+      <c r="AU137" s="22" t="n"/>
+      <c r="AW137" s="0" t="n"/>
+      <c r="BA137" s="22" t="n"/>
+      <c r="BC137" s="0" t="n"/>
+      <c r="BG137" s="22" t="n"/>
+      <c r="BI137" s="0" t="n"/>
+      <c r="BM137" s="22" t="n"/>
+      <c r="BS137" s="22" t="n"/>
+      <c r="BY137" s="22" t="n"/>
+      <c r="CE137" s="22" t="n"/>
+      <c r="CG137" s="0" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="0" t="inlineStr">
@@ -26631,144 +26549,78 @@
           <t>java.lang.Object</t>
         </is>
       </c>
+      <c r="C138" t="b">
+        <v>0</v>
+      </c>
       <c r="D138" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="G138" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="R138" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="S138" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="T138" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="U138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="V138" s="0" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E138" s="22" t="n"/>
+      <c r="G138" s="0" t="n"/>
+      <c r="K138" s="22" t="n"/>
+      <c r="Q138" s="22" t="n"/>
+      <c r="R138" s="0" t="n"/>
+      <c r="S138" s="0" t="n"/>
+      <c r="T138" s="0" t="n"/>
+      <c r="U138" s="0" t="n"/>
+      <c r="V138" s="0" t="n"/>
+      <c r="W138" s="22" t="n"/>
       <c r="AD138" s="0" t="inlineStr">
         <is>
           <t>linestring</t>
         </is>
       </c>
-      <c r="AE138" s="0" t="inlineStr">
+      <c r="AE138" s="0" t="n"/>
+      <c r="AF138" s="0" t="inlineStr">
         <is>
           <t>linestring</t>
         </is>
       </c>
-      <c r="AF138" s="0" t="inlineStr">
+      <c r="AG138" s="0" t="n"/>
+      <c r="AH138" s="0" t="n"/>
+      <c r="AI138" s="22" t="n"/>
+      <c r="AJ138" s="0" t="n"/>
+      <c r="AK138" s="0" t="n"/>
+      <c r="AL138" s="0" t="n"/>
+      <c r="AM138" s="0" t="n"/>
+      <c r="AN138" s="0" t="n"/>
+      <c r="AP138" s="0" t="inlineStr">
         <is>
           <t>linestring</t>
         </is>
       </c>
-      <c r="AG138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ138" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AK138" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AL138" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AM138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP138" s="0" t="inlineStr">
+      <c r="AQ138" s="0" t="n"/>
+      <c r="AR138" s="0" t="inlineStr">
         <is>
           <t>linestring</t>
         </is>
       </c>
-      <c r="AQ138" s="0" t="inlineStr">
+      <c r="AS138" s="0" t="n"/>
+      <c r="AT138" s="0" t="n"/>
+      <c r="AU138" s="22" t="n"/>
+      <c r="AW138" s="0" t="n"/>
+      <c r="BA138" s="22" t="n"/>
+      <c r="BB138" s="0" t="n"/>
+      <c r="BC138" s="0" t="n"/>
+      <c r="BG138" s="22" t="n"/>
+      <c r="BH138" s="0" t="n"/>
+      <c r="BI138" s="0" t="n"/>
+      <c r="BM138" s="22" t="n"/>
+      <c r="BS138" s="22" t="n"/>
+      <c r="BY138" s="22" t="n"/>
+      <c r="CF138" s="0" t="inlineStr">
         <is>
           <t>linestring</t>
         </is>
       </c>
-      <c r="AR138" s="0" t="inlineStr">
+      <c r="CG138" s="0" t="n"/>
+      <c r="CH138" s="0" t="inlineStr">
         <is>
           <t>linestring</t>
         </is>
       </c>
-      <c r="AS138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW138" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="BB138" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BC138" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BH138" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BI138" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="CF138" s="0" t="inlineStr">
-        <is>
-          <t>linestring</t>
-        </is>
-      </c>
-      <c r="CG138" s="0" t="inlineStr">
-        <is>
-          <t>linestring</t>
-        </is>
-      </c>
-      <c r="CH138" s="0" t="inlineStr">
-        <is>
-          <t>linestring</t>
-        </is>
-      </c>
-      <c r="CI138" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ138" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI138" s="0" t="n"/>
+      <c r="CJ138" s="0" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="0" t="inlineStr">
@@ -26781,107 +26633,69 @@
           <t>java.lang.Object</t>
         </is>
       </c>
+      <c r="C139" t="b">
+        <v>0</v>
+      </c>
       <c r="D139" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="G139" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="R139" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="S139" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E139" s="22" t="n"/>
+      <c r="G139" s="0" t="n"/>
+      <c r="K139" s="22" t="n"/>
+      <c r="Q139" s="22" t="n"/>
+      <c r="R139" s="0" t="n"/>
+      <c r="S139" s="0" t="n"/>
+      <c r="W139" s="22" t="n"/>
       <c r="AD139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AE139" s="0" t="inlineStr">
+      <c r="AE139" s="0" t="n"/>
+      <c r="AF139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AF139" s="0" t="inlineStr">
+      <c r="AG139" s="0" t="n"/>
+      <c r="AH139" s="0" t="n"/>
+      <c r="AI139" s="22" t="n"/>
+      <c r="AK139" s="0" t="n"/>
+      <c r="AP139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AG139" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH139" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK139" s="0" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="AP139" s="0" t="inlineStr">
+      <c r="AQ139" s="0" t="n"/>
+      <c r="AR139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AQ139" s="0" t="inlineStr">
+      <c r="AS139" s="0" t="n"/>
+      <c r="AT139" s="0" t="n"/>
+      <c r="AU139" s="22" t="n"/>
+      <c r="AW139" s="0" t="n"/>
+      <c r="BA139" s="22" t="n"/>
+      <c r="BC139" s="0" t="n"/>
+      <c r="BG139" s="22" t="n"/>
+      <c r="BI139" s="0" t="n"/>
+      <c r="BM139" s="22" t="n"/>
+      <c r="BS139" s="22" t="n"/>
+      <c r="BY139" s="22" t="n"/>
+      <c r="CF139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AR139" s="0" t="inlineStr">
+      <c r="CG139" s="0" t="n"/>
+      <c r="CH139" s="0" t="inlineStr">
         <is>
           <t>multipoint</t>
         </is>
       </c>
-      <c r="AS139" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT139" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW139" s="0" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="BC139" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="BI139" s="0" t="inlineStr">
-        <is>
-          <t>nvarchar(max)</t>
-        </is>
-      </c>
-      <c r="CF139" s="0" t="inlineStr">
-        <is>
-          <t>multipoint</t>
-        </is>
-      </c>
-      <c r="CG139" s="0" t="inlineStr">
-        <is>
-          <t>multipoint</t>
-        </is>
-      </c>
-      <c r="CH139" s="0" t="inlineStr">
-        <is>
-          <t>multipoint</t>
-        </is>
-      </c>
-      <c r="CI139" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ139" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI139" s="0" t="n"/>
+      <c r="CJ139" s="0" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="0" t="inlineStr">
@@ -26894,69 +26708,62 @@
           <t>java.lang.Object</t>
         </is>
       </c>
+      <c r="C140" t="b">
+        <v>0</v>
+      </c>
+      <c r="D140" t="b">
+        <v>0</v>
+      </c>
+      <c r="E140" s="22" t="n"/>
+      <c r="K140" s="22" t="n"/>
+      <c r="Q140" s="22" t="n"/>
+      <c r="W140" s="22" t="n"/>
       <c r="AD140" s="0" t="inlineStr">
         <is>
           <t>multilinestring</t>
         </is>
       </c>
-      <c r="AE140" s="0" t="inlineStr">
+      <c r="AE140" s="0" t="n"/>
+      <c r="AF140" s="0" t="inlineStr">
         <is>
           <t>multilinestring</t>
         </is>
       </c>
-      <c r="AF140" s="0" t="inlineStr">
+      <c r="AG140" s="0" t="n"/>
+      <c r="AH140" s="0" t="n"/>
+      <c r="AI140" s="22" t="n"/>
+      <c r="AP140" s="0" t="inlineStr">
         <is>
           <t>multilinestring</t>
         </is>
       </c>
-      <c r="AG140" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH140" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP140" s="0" t="inlineStr">
+      <c r="AQ140" s="0" t="n"/>
+      <c r="AR140" s="0" t="inlineStr">
         <is>
           <t>multilinestring</t>
         </is>
       </c>
-      <c r="AQ140" s="0" t="inlineStr">
+      <c r="AS140" s="0" t="n"/>
+      <c r="AT140" s="0" t="n"/>
+      <c r="AU140" s="22" t="n"/>
+      <c r="BA140" s="22" t="n"/>
+      <c r="BG140" s="22" t="n"/>
+      <c r="BM140" s="22" t="n"/>
+      <c r="BS140" s="22" t="n"/>
+      <c r="BY140" s="22" t="n"/>
+      <c r="CF140" s="0" t="inlineStr">
         <is>
           <t>multilinestring</t>
         </is>
       </c>
-      <c r="AR140" s="0" t="inlineStr">
+      <c r="CG140" s="0" t="n"/>
+      <c r="CH140" s="0" t="inlineStr">
         <is>
           <t>multilinestring</t>
         </is>
       </c>
-      <c r="AS140" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT140" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF140" s="0" t="inlineStr">
-        <is>
-          <t>multilinestring</t>
-        </is>
-      </c>
-      <c r="CG140" s="0" t="inlineStr">
-        <is>
-          <t>multilinestring</t>
-        </is>
-      </c>
-      <c r="CH140" s="0" t="inlineStr">
-        <is>
-          <t>multilinestring</t>
-        </is>
-      </c>
-      <c r="CI140" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ140" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI140" s="0" t="n"/>
+      <c r="CJ140" s="0" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="0" t="inlineStr">
@@ -26969,69 +26776,62 @@
           <t>java.lang.Object</t>
         </is>
       </c>
+      <c r="C141" t="b">
+        <v>0</v>
+      </c>
+      <c r="D141" t="b">
+        <v>0</v>
+      </c>
+      <c r="E141" s="22" t="n"/>
+      <c r="K141" s="22" t="n"/>
+      <c r="Q141" s="22" t="n"/>
+      <c r="W141" s="22" t="n"/>
       <c r="AD141" s="0" t="inlineStr">
         <is>
           <t>multipolygon</t>
         </is>
       </c>
-      <c r="AE141" s="0" t="inlineStr">
+      <c r="AE141" s="0" t="n"/>
+      <c r="AF141" s="0" t="inlineStr">
         <is>
           <t>multipolygon</t>
         </is>
       </c>
-      <c r="AF141" s="0" t="inlineStr">
+      <c r="AG141" s="0" t="n"/>
+      <c r="AH141" s="0" t="n"/>
+      <c r="AI141" s="22" t="n"/>
+      <c r="AP141" s="0" t="inlineStr">
         <is>
           <t>multipolygon</t>
         </is>
       </c>
-      <c r="AG141" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH141" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP141" s="0" t="inlineStr">
+      <c r="AQ141" s="0" t="n"/>
+      <c r="AR141" s="0" t="inlineStr">
         <is>
           <t>multipolygon</t>
         </is>
       </c>
-      <c r="AQ141" s="0" t="inlineStr">
+      <c r="AS141" s="0" t="n"/>
+      <c r="AT141" s="0" t="n"/>
+      <c r="AU141" s="22" t="n"/>
+      <c r="BA141" s="22" t="n"/>
+      <c r="BG141" s="22" t="n"/>
+      <c r="BM141" s="22" t="n"/>
+      <c r="BS141" s="22" t="n"/>
+      <c r="BY141" s="22" t="n"/>
+      <c r="CF141" s="0" t="inlineStr">
         <is>
           <t>multipolygon</t>
         </is>
       </c>
-      <c r="AR141" s="0" t="inlineStr">
+      <c r="CG141" s="0" t="n"/>
+      <c r="CH141" s="0" t="inlineStr">
         <is>
           <t>multipolygon</t>
         </is>
       </c>
-      <c r="AS141" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT141" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF141" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="CG141" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="CH141" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="CI141" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ141" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI141" s="0" t="n"/>
+      <c r="CJ141" s="0" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="0" t="inlineStr">
@@ -27044,69 +26844,62 @@
           <t>java.lang.Object</t>
         </is>
       </c>
+      <c r="C142" t="b">
+        <v>0</v>
+      </c>
+      <c r="D142" t="b">
+        <v>0</v>
+      </c>
+      <c r="E142" s="22" t="n"/>
+      <c r="K142" s="22" t="n"/>
+      <c r="Q142" s="22" t="n"/>
+      <c r="W142" s="22" t="n"/>
       <c r="AD142" s="0" t="inlineStr">
         <is>
           <t>geometrycollection</t>
         </is>
       </c>
-      <c r="AE142" s="0" t="inlineStr">
+      <c r="AE142" s="0" t="n"/>
+      <c r="AF142" s="0" t="inlineStr">
         <is>
           <t>geometrycollection</t>
         </is>
       </c>
-      <c r="AF142" s="0" t="inlineStr">
+      <c r="AG142" s="0" t="n"/>
+      <c r="AH142" s="0" t="n"/>
+      <c r="AI142" s="22" t="n"/>
+      <c r="AP142" s="0" t="inlineStr">
         <is>
           <t>geometrycollection</t>
         </is>
       </c>
-      <c r="AG142" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH142" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP142" s="0" t="inlineStr">
+      <c r="AQ142" s="0" t="n"/>
+      <c r="AR142" s="0" t="inlineStr">
         <is>
           <t>geometrycollection</t>
         </is>
       </c>
-      <c r="AQ142" s="0" t="inlineStr">
+      <c r="AS142" s="0" t="n"/>
+      <c r="AT142" s="0" t="n"/>
+      <c r="AU142" s="22" t="n"/>
+      <c r="BA142" s="22" t="n"/>
+      <c r="BG142" s="22" t="n"/>
+      <c r="BM142" s="22" t="n"/>
+      <c r="BS142" s="22" t="n"/>
+      <c r="BY142" s="22" t="n"/>
+      <c r="CF142" s="0" t="inlineStr">
         <is>
           <t>geometrycollection</t>
         </is>
       </c>
-      <c r="AR142" s="0" t="inlineStr">
+      <c r="CG142" s="0" t="n"/>
+      <c r="CH142" s="0" t="inlineStr">
         <is>
           <t>geometrycollection</t>
         </is>
       </c>
-      <c r="AS142" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT142" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF142" s="0" t="inlineStr">
-        <is>
-          <t>geometrycollection</t>
-        </is>
-      </c>
-      <c r="CG142" s="0" t="inlineStr">
-        <is>
-          <t>geometrycollection</t>
-        </is>
-      </c>
-      <c r="CH142" s="0" t="inlineStr">
-        <is>
-          <t>geometrycollection</t>
-        </is>
-      </c>
-      <c r="CI142" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ142" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI142" s="0" t="n"/>
+      <c r="CJ142" s="0" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="0" t="inlineStr">
@@ -27119,111 +26912,72 @@
           <t>java.lang.Object</t>
         </is>
       </c>
-      <c r="AD143" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="AE143" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-      <c r="AF143" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="AG143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH143" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="C143" t="b">
+        <v>0</v>
+      </c>
+      <c r="D143" t="b">
+        <v>0</v>
+      </c>
+      <c r="E143" s="22" t="n"/>
+      <c r="K143" s="22" t="n"/>
+      <c r="Q143" s="22" t="n"/>
+      <c r="W143" s="22" t="n"/>
+      <c r="AC143" s="22" t="n"/>
+      <c r="AD143" s="0" t="n"/>
+      <c r="AE143" s="0" t="n"/>
+      <c r="AF143" s="0" t="n"/>
+      <c r="AG143" s="0" t="n"/>
+      <c r="AH143" s="0" t="n"/>
+      <c r="AI143" s="22" t="n"/>
       <c r="AP143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="AQ143" s="0" t="inlineStr">
+      <c r="AQ143" s="0" t="n"/>
+      <c r="AR143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="AR143" s="0" t="inlineStr">
+      <c r="AS143" s="0" t="n"/>
+      <c r="AT143" s="0" t="n"/>
+      <c r="AU143" s="22" t="n"/>
+      <c r="BB143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="AS143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB143" s="0" t="inlineStr">
+      <c r="BC143" s="0" t="n"/>
+      <c r="BD143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BC143" s="0" t="inlineStr">
+      <c r="BE143" s="0" t="n"/>
+      <c r="BF143" s="0" t="n"/>
+      <c r="BH143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BD143" s="0" t="inlineStr">
+      <c r="BI143" s="0" t="n"/>
+      <c r="BJ143" s="0" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="BE143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH143" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BI143" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BJ143" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BK143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF143" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="CG143" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-      <c r="CH143" s="0" t="inlineStr">
-        <is>
-          <t>multipolygon</t>
-        </is>
-      </c>
-      <c r="CI143" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ143" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="BK143" s="0" t="n"/>
+      <c r="BL143" s="0" t="n"/>
+      <c r="BM143" s="22" t="n"/>
+      <c r="BS143" s="22" t="n"/>
+      <c r="BY143" s="22" t="n"/>
+      <c r="CE143" s="22" t="n"/>
+      <c r="CF143" s="0" t="n"/>
+      <c r="CG143" s="0" t="n"/>
+      <c r="CH143" s="0" t="n"/>
+      <c r="CI143" s="0" t="n"/>
+      <c r="CJ143" s="0" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
@@ -27236,69 +26990,48 @@
           <t>java.lang.String</t>
         </is>
       </c>
-      <c r="AD144" s="0" t="inlineStr">
-        <is>
-          <t>geometrycollection</t>
-        </is>
-      </c>
-      <c r="AE144" s="0" t="inlineStr">
-        <is>
-          <t>varchar(15)</t>
-        </is>
-      </c>
-      <c r="AF144" s="0" t="inlineStr">
-        <is>
-          <t>geometrycollection</t>
-        </is>
-      </c>
-      <c r="AG144" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH144" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP144" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AQ144" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AR144" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AS144" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT144" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="C144" t="b">
+        <v>0</v>
+      </c>
+      <c r="D144" t="b">
+        <v>0</v>
+      </c>
+      <c r="E144" s="22" t="n"/>
+      <c r="K144" s="22" t="n"/>
+      <c r="Q144" s="22" t="n"/>
+      <c r="W144" s="22" t="n"/>
+      <c r="AC144" s="22" t="n"/>
+      <c r="AD144" s="0" t="n"/>
+      <c r="AE144" s="0" t="n"/>
+      <c r="AF144" s="0" t="n"/>
+      <c r="AG144" s="0" t="n"/>
+      <c r="AH144" s="0" t="n"/>
+      <c r="AI144" s="22" t="n"/>
+      <c r="AO144" s="22" t="n"/>
+      <c r="AP144" s="0" t="n"/>
+      <c r="AQ144" s="0" t="n"/>
+      <c r="AR144" s="0" t="n"/>
+      <c r="AS144" s="0" t="n"/>
+      <c r="AT144" s="0" t="n"/>
+      <c r="AU144" s="22" t="n"/>
+      <c r="BA144" s="22" t="n"/>
+      <c r="BG144" s="22" t="n"/>
+      <c r="BM144" s="22" t="n"/>
+      <c r="BS144" s="22" t="n"/>
+      <c r="BY144" s="22" t="n"/>
       <c r="CF144" s="0" t="inlineStr">
         <is>
           <t>inet4</t>
         </is>
       </c>
-      <c r="CG144" s="0" t="inlineStr">
+      <c r="CG144" s="0" t="n"/>
+      <c r="CH144" s="0" t="inlineStr">
         <is>
           <t>inet4</t>
         </is>
       </c>
-      <c r="CH144" s="0" t="inlineStr">
-        <is>
-          <t>inet4</t>
-        </is>
-      </c>
-      <c r="CI144" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ144" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI144" s="0" t="n"/>
+      <c r="CJ144" s="0" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
@@ -27311,95 +27044,54 @@
           <t>java.lang.String</t>
         </is>
       </c>
-      <c r="AE145" s="0" t="inlineStr">
-        <is>
-          <t>varchar(45)</t>
-        </is>
-      </c>
-      <c r="AP145" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AQ145" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AR145" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AS145" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT145" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB145" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BC145" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BD145" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BE145" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF145" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH145" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BI145" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BJ145" s="0" t="inlineStr">
-        <is>
-          <t>geography</t>
-        </is>
-      </c>
-      <c r="BK145" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL145" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="C145" t="b">
+        <v>0</v>
+      </c>
+      <c r="D145" t="b">
+        <v>0</v>
+      </c>
+      <c r="E145" s="22" t="n"/>
+      <c r="K145" s="22" t="n"/>
+      <c r="Q145" s="22" t="n"/>
+      <c r="W145" s="22" t="n"/>
+      <c r="AC145" s="22" t="n"/>
+      <c r="AE145" s="0" t="n"/>
+      <c r="AI145" s="22" t="n"/>
+      <c r="AO145" s="22" t="n"/>
+      <c r="AP145" s="0" t="n"/>
+      <c r="AQ145" s="0" t="n"/>
+      <c r="AR145" s="0" t="n"/>
+      <c r="AS145" s="0" t="n"/>
+      <c r="AT145" s="0" t="n"/>
+      <c r="AU145" s="22" t="n"/>
+      <c r="BA145" s="22" t="n"/>
+      <c r="BB145" s="0" t="n"/>
+      <c r="BC145" s="0" t="n"/>
+      <c r="BD145" s="0" t="n"/>
+      <c r="BE145" s="0" t="n"/>
+      <c r="BF145" s="0" t="n"/>
+      <c r="BG145" s="22" t="n"/>
+      <c r="BH145" s="0" t="n"/>
+      <c r="BI145" s="0" t="n"/>
+      <c r="BJ145" s="0" t="n"/>
+      <c r="BK145" s="0" t="n"/>
+      <c r="BL145" s="0" t="n"/>
+      <c r="BM145" s="22" t="n"/>
+      <c r="BS145" s="22" t="n"/>
+      <c r="BY145" s="22" t="n"/>
       <c r="CF145" s="0" t="inlineStr">
         <is>
           <t>inet6</t>
         </is>
       </c>
-      <c r="CG145" s="0" t="inlineStr">
+      <c r="CG145" s="0" t="n"/>
+      <c r="CH145" s="0" t="inlineStr">
         <is>
           <t>inet6</t>
         </is>
       </c>
-      <c r="CH145" s="0" t="inlineStr">
-        <is>
-          <t>inet6</t>
-        </is>
-      </c>
-      <c r="CI145" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ145" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="CI145" s="0" t="n"/>
+      <c r="CJ145" s="0" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
@@ -27412,233 +27104,131 @@
           <t>java.lang.Object</t>
         </is>
       </c>
-      <c r="AE146" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
+      <c r="C146" t="b">
+        <v>0</v>
+      </c>
+      <c r="D146" t="b">
+        <v>0</v>
+      </c>
+      <c r="E146" s="22" t="n"/>
+      <c r="K146" s="22" t="n"/>
+      <c r="Q146" s="22" t="n"/>
+      <c r="W146" s="22" t="n"/>
+      <c r="AC146" s="22" t="n"/>
+      <c r="AE146" s="0" t="n"/>
       <c r="AJ146" s="0" t="inlineStr">
         <is>
           <t>sdo_geometry</t>
         </is>
       </c>
-      <c r="AK146" s="0" t="inlineStr">
+      <c r="AK146" s="0" t="n"/>
+      <c r="AL146" s="0" t="inlineStr">
         <is>
           <t>sdo_geometry</t>
         </is>
       </c>
-      <c r="AL146" s="0" t="inlineStr">
-        <is>
-          <t>sdo_geometry</t>
-        </is>
-      </c>
-      <c r="AM146" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN146" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP146" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AQ146" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-      <c r="AR146" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AS146" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT146" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF146" s="0" t="inlineStr">
-        <is>
-          <t>inet4</t>
-        </is>
-      </c>
-      <c r="CG146" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-      <c r="CH146" s="0" t="inlineStr">
-        <is>
-          <t>inet4</t>
-        </is>
-      </c>
-      <c r="CI146" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ146" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="AM146" s="0" t="n"/>
+      <c r="AN146" s="0" t="n"/>
+      <c r="AO146" s="22" t="n"/>
+      <c r="AP146" s="0" t="n"/>
+      <c r="AQ146" s="0" t="n"/>
+      <c r="AR146" s="0" t="n"/>
+      <c r="AS146" s="0" t="n"/>
+      <c r="AT146" s="0" t="n"/>
+      <c r="AU146" s="22" t="n"/>
+      <c r="BA146" s="22" t="n"/>
+      <c r="BG146" s="22" t="n"/>
+      <c r="BM146" s="22" t="n"/>
+      <c r="BS146" s="22" t="n"/>
+      <c r="BY146" s="22" t="n"/>
+      <c r="CE146" s="22" t="n"/>
+      <c r="CF146" s="0" t="n"/>
+      <c r="CG146" s="0" t="n"/>
+      <c r="CH146" s="0" t="n"/>
+      <c r="CI146" s="0" t="n"/>
+      <c r="CJ146" s="0" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t>inet6</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="B147" s="0" t="inlineStr">
         <is>
-          <t>java.lang.String</t>
-        </is>
-      </c>
-      <c r="AE147" s="0" t="inlineStr">
-        <is>
-          <t>varchar(45)</t>
+          <t>java.lang.Object</t>
+        </is>
+      </c>
+      <c r="C147" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="D147" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="F147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="H147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="K147" s="22" t="n"/>
+      <c r="Q147" s="22" t="n"/>
+      <c r="W147" s="22" t="n"/>
+      <c r="AD147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AF147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AJ147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AL147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
         </is>
       </c>
       <c r="AP147" s="0" t="inlineStr">
         <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AQ147" s="0" t="inlineStr">
-        <is>
-          <t>inet</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="AR147" s="0" t="inlineStr">
         <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="AS147" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT147" s="0" t="n">
-        <v>0</v>
-      </c>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="AU147" s="22" t="n"/>
+      <c r="BB147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="BD147" s="0" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="BG147" s="22" t="n"/>
+      <c r="BM147" s="22" t="n"/>
+      <c r="BS147" s="22" t="n"/>
+      <c r="BY147" s="22" t="n"/>
       <c r="CF147" s="0" t="inlineStr">
         <is>
-          <t>inet6</t>
-        </is>
-      </c>
-      <c r="CG147" s="0" t="inlineStr">
-        <is>
-          <t>inet6</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="CH147" s="0" t="inlineStr">
-        <is>
-          <t>inet6</t>
-        </is>
-      </c>
-      <c r="CI147" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="CJ147" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="0" t="inlineStr">
-        <is>
-          <t>sdo_geometry</t>
-        </is>
-      </c>
-      <c r="B148" s="0" t="inlineStr">
-        <is>
-          <t>java.lang.Object</t>
-        </is>
-      </c>
-      <c r="AE148" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-      <c r="AJ148" s="0" t="inlineStr">
-        <is>
-          <t>sdo_geometry</t>
-        </is>
-      </c>
-      <c r="AK148" s="0" t="inlineStr">
-        <is>
-          <t>sdo_geometry</t>
-        </is>
-      </c>
-      <c r="AL148" s="0" t="inlineStr">
-        <is>
-          <t>sdo_geometry</t>
-        </is>
-      </c>
-      <c r="AM148" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN148" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ148" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-      <c r="CG148" s="0" t="inlineStr">
-        <is>
-          <t>geometry</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>java.lang.Object</t>
-        </is>
-      </c>
-      <c r="C149" t="b">
-        <v>1</v>
-      </c>
-      <c r="D149" t="b">
-        <v>0</v>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="K149" s="22" t="n"/>
-      <c r="Q149" s="22" t="n"/>
-      <c r="W149" s="22" t="n"/>
-      <c r="AD149" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="AJ149" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="AP149" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="AU149" s="22" t="n"/>
-      <c r="BB149" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="BG149" s="22" t="n"/>
-      <c r="BM149" s="22" t="n"/>
-      <c r="BS149" s="22" t="n"/>
-      <c r="BY149" s="22" t="n"/>
-      <c r="CF149" t="inlineStr">
         <is>
           <t>vector</t>
         </is>

</xml_diff>